<commit_message>
data: W24 SOH refreshed to Jun 13 (Saturday point-in-time)
Vendor SOH (SP-API) re-pulled now that Amazon has published the
Saturday Jun 13 row.  Inventory now matches sales on the full
Sun-Sat W24 window (Jun 7-13).

W24 1P SOH:
  Audio Array  7,603 units / Rs 1.35 Cr
  Tonor          686 units / Rs 7.26 L
  White Mulberry 231 units / Rs 0       (WM ASINs still untagged in master)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/inventory/Week 24/Tonor/Vendor SOH (SP-API).xlsx
+++ b/data/raw/inventory/Week 24/Tonor/Vendor SOH (SP-API).xlsx
@@ -518,12 +518,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FBA77105</t>
+          <t>FBA79113</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>B089FVQD3Z</t>
+          <t>B0BTCXQQ6M</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -533,25 +533,25 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>TC310</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Boom Arm Kit</t>
+          <t>Tripod - RGB</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>1477</v>
+        <v>1206</v>
       </c>
       <c r="I2" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -563,32 +563,32 @@
         <v>24</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P2" t="n">
-        <v>5718.87</v>
+        <v>28018.53</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FBA77116</t>
+          <t>FBA77117</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B0BBL47VR5</t>
+          <t>B078WNW4YW</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -598,25 +598,25 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>TC40S</t>
+          <t>S20</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Boom Arm Kit - USB - RGB</t>
+          <t>Microphone Isolation Shield</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>1930</v>
+        <v>1174</v>
       </c>
       <c r="I3" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -628,32 +628,32 @@
         <v>24</v>
       </c>
       <c r="M3" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="N3" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="O3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P3" t="n">
-        <v>10345.5</v>
+        <v>46464.37</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FBA79696</t>
+          <t>FBA77113</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B0CQX3VB1R</t>
+          <t>B01ISNU3X4</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>TD310+</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -673,15 +673,15 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Hand held Mic + Boom Arm</t>
+          <t>Hand held Mic</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>927</v>
+        <v>848</v>
       </c>
       <c r="I4" t="n">
-        <v>31</v>
+        <v>248</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -693,32 +693,32 @@
         <v>24</v>
       </c>
       <c r="M4" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O4" t="n">
         <v>5</v>
       </c>
       <c r="P4" t="n">
-        <v>54757.56</v>
+        <v>313569.29</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FBA77106</t>
+          <t>FBA79111</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>B082W4B7SX</t>
+          <t>B0BRKFP94K</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -728,25 +728,25 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>TD510</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Dynamic Microphone</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Boom Arm Kit</t>
+          <t>USB/XLR Mic</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>1164</v>
+        <v>2412</v>
       </c>
       <c r="I5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -758,32 +758,32 @@
         <v>24</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P5" t="n">
-        <v>8260.200000000001</v>
+        <v>21992.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FBA77110</t>
+          <t>FBA79576</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B08NDB5NWP</t>
+          <t>B0BRCR2QQ7</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -793,25 +793,25 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>TM20</t>
+          <t>TC30S+</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Conference Microphone</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Wired</t>
+          <t>Boom Arm Kit + RGB</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>1695</v>
+        <v>1749</v>
       </c>
       <c r="I6" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -823,32 +823,32 @@
         <v>24</v>
       </c>
       <c r="M6" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>57286.92</v>
+        <v>12331.21</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FBA79577</t>
+          <t>FBA79114</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>B0CSCT63BL</t>
+          <t>B0CCV74CL7</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -858,25 +858,25 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>TM310</t>
+          <t>TC310+</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Conference Microphone</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Wired</t>
+          <t>Boom Arm Kit - USB - RGB</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>965</v>
+        <v>1689</v>
       </c>
       <c r="I7" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -888,32 +888,32 @@
         <v>24</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P7" t="n">
-        <v>10416.65</v>
+        <v>30197.39</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FBA77114</t>
+          <t>FBA79116</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>B07TSN2H9D</t>
+          <t>B0BYHHSLPC</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TC-2030</t>
+          <t>TC-777 PRO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -933,15 +933,15 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Boom Arm Kit - USB</t>
+          <t>Tripod - RGB</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>4423</v>
+        <v>1086</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -953,30 +953,32 @@
         <v>24</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="P8" t="n">
+        <v>32632.59</v>
+      </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FBA79578</t>
+          <t>FBA79579</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>B0CFKZ72N7</t>
+          <t>B0CQX4GVSB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -986,7 +988,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1001,7 +1003,7 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>1688</v>
+        <v>1244</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1027,19 +1029,19 @@
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FBA79112</t>
+          <t>FBA77110</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>B0BRKDLXCD</t>
+          <t>B08NDB5NWP</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1049,25 +1051,25 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>TM20</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Conference Microphone</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Boom Arm - RGB</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>2412</v>
+        <v>1695</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1079,7 +1081,7 @@
         <v>24</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -1087,22 +1089,24 @@
       <c r="O10" t="n">
         <v>0</v>
       </c>
-      <c r="P10" t="inlineStr"/>
+      <c r="P10" t="n">
+        <v>55165.18</v>
+      </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FBA79114</t>
+          <t>FBA79575</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>B0CCV74CL7</t>
+          <t>B0BG8CJXHH</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1112,7 +1116,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>TC310+</t>
+          <t>TC30+</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1122,15 +1126,15 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Boom Arm Kit - USB - RGB</t>
+          <t>Boom Arm Kit</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>1689</v>
+        <v>1568</v>
       </c>
       <c r="I11" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1142,32 +1146,32 @@
         <v>24</v>
       </c>
       <c r="M11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="O11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>32713.83</v>
+        <v>22018.71</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FBK77102</t>
+          <t>FBA77105</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>B07GVGMW59</t>
+          <t>B089FVQD3Z</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1177,25 +1181,25 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>G11</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Conference Microphone</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Wired</t>
+          <t>Boom Arm Kit</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>1108</v>
+        <v>1477</v>
       </c>
       <c r="I12" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1207,32 +1211,32 @@
         <v>24</v>
       </c>
       <c r="M12" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>94093.78999999999</v>
+        <v>5718.87</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FBA77103</t>
+          <t>FBA79577</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>B09Z5Q194D</t>
+          <t>B0CSCT63BL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1242,25 +1246,25 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ORCA001</t>
+          <t>TM310</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Conference Microphone</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Stand</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>2412</v>
+        <v>965</v>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1275,29 +1279,29 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>7528.69</v>
+        <v>10416.65</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FBA77101</t>
+          <t>FBA79574</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>B07WLWN2ZT</t>
+          <t>B0B4WTHLX5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1307,7 +1311,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>TC-777</t>
+          <t>TC30S</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1317,15 +1321,15 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Tripod</t>
+          <t>Tripod+RGB</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>1206</v>
+        <v>1448</v>
       </c>
       <c r="I14" t="n">
-        <v>41</v>
+        <v>4</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1337,32 +1341,32 @@
         <v>24</v>
       </c>
       <c r="M14" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N14" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>70180.48</v>
+        <v>8298.77</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FBA79575</t>
+          <t>FBA79582</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>B0BG8CJXHH</t>
+          <t>B0CCVBQRFX</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1372,25 +1376,25 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>TC30+</t>
+          <t>TD510+</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Dynamic Microphone</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Boom Arm Kit</t>
+          <t>Hand held Mic + Boom Arm</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>1568</v>
+        <v>3491</v>
       </c>
       <c r="I15" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1405,29 +1409,29 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>22018.71</v>
+        <v>4334.39</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FBA79579</t>
+          <t>FBA79697</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>B0CQX4GVSB</t>
+          <t>B0CQX4K9P5</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1437,7 +1441,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>TD310</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1447,15 +1451,15 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Hand held Mic</t>
+          <t>Hand held Mic + Stand</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>1244</v>
+        <v>790</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1473,24 +1477,26 @@
         <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="P16" t="n">
+        <v>188582.58</v>
+      </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FBA79697</t>
+          <t>FBA77106</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>B0CQX4K9P5</t>
+          <t>B082W4B7SX</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1500,25 +1506,25 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TD310</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Dynamic Microphone</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Hand held Mic + Stand</t>
+          <t>Boom Arm Kit</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>790</v>
+        <v>1164</v>
       </c>
       <c r="I17" t="n">
-        <v>114</v>
+        <v>5</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1536,26 +1542,26 @@
         <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P17" t="n">
-        <v>191950.12</v>
+        <v>8260.200000000001</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FBA77113</t>
+          <t>FBA79696</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>B01ISNU3X4</t>
+          <t>B0CQX3VB1R</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1565,7 +1571,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>TD310+</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1575,15 +1581,15 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Hand held Mic</t>
+          <t>Hand held Mic + Boom Arm</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>848</v>
+        <v>927</v>
       </c>
       <c r="I18" t="n">
-        <v>248</v>
+        <v>31</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1595,32 +1601,32 @@
         <v>24</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="N18" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="O18" t="n">
         <v>5</v>
       </c>
       <c r="P18" t="n">
-        <v>313535.6</v>
+        <v>54757.56</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FBA79574</t>
+          <t>FBA79585</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>B0B4WTHLX5</t>
+          <t>B0CFKHCQ8W</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1630,25 +1636,25 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>TC30S</t>
+          <t>T20LP</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Tripod+RGB</t>
+          <t>Low Profile Boom Arm</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>1448</v>
+        <v>845</v>
       </c>
       <c r="I19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1663,29 +1669,29 @@
         <v>2</v>
       </c>
       <c r="N19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P19" t="n">
-        <v>8298.77</v>
+        <v>4384.04</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FBA77117</t>
+          <t>FBA77103</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>B078WNW4YW</t>
+          <t>B09Z5Q194D</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1695,25 +1701,25 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>S20</t>
+          <t>ORCA001</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Microphone Isolation Shield</t>
+          <t>Stand</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>1174</v>
+        <v>2412</v>
       </c>
       <c r="I20" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1725,32 +1731,32 @@
         <v>24</v>
       </c>
       <c r="M20" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="O20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>46464.37</v>
+        <v>7528.69</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FBA79576</t>
+          <t>FBA79115</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>B0BRCR2QQ7</t>
+          <t>B0C8JDHLX9</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1760,25 +1766,25 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TC30S+</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Boom Arm Kit + RGB</t>
+          <t>Boom Arm Kit</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>1749</v>
+        <v>603</v>
       </c>
       <c r="I21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1790,32 +1796,32 @@
         <v>24</v>
       </c>
       <c r="M21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O21" t="n">
         <v>0</v>
       </c>
       <c r="P21" t="n">
-        <v>12331.21</v>
+        <v>2401.47</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FBA79116</t>
+          <t>FBA77114</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>B0BYHHSLPC</t>
+          <t>B07TSN2H9D</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1825,7 +1831,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>TC-777 PRO</t>
+          <t>TC-2030</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1835,15 +1841,15 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Tripod - RGB</t>
+          <t>Boom Arm Kit - USB</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>1086</v>
+        <v>4423</v>
       </c>
       <c r="I22" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1855,32 +1861,30 @@
         <v>24</v>
       </c>
       <c r="M22" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O22" t="n">
-        <v>14</v>
-      </c>
-      <c r="P22" t="n">
-        <v>41388.38</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FBA77115</t>
+          <t>FBA77104</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>B08V1JS3NY</t>
+          <t>B089SJGQBH</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1890,7 +1894,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>TC40</t>
+          <t>TC20</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1900,15 +1904,15 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Boom Arm Kit - USB</t>
+          <t>Boom Arm Kit - XLR</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>1930</v>
+        <v>3015</v>
       </c>
       <c r="I23" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1920,32 +1924,30 @@
         <v>24</v>
       </c>
       <c r="M23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>1</v>
-      </c>
-      <c r="P23" t="n">
-        <v>22543.15</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FBA79115</t>
+          <t>FBA79578</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>B0C8JDHLX9</t>
+          <t>B0CFKZ72N7</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1955,25 +1957,25 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>T10</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Dynamic Microphone</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Boom Arm Kit</t>
+          <t>Hand held Mic</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>603</v>
+        <v>1688</v>
       </c>
       <c r="I24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1988,29 +1990,27 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
-      <c r="P24" t="n">
-        <v>2401.47</v>
-      </c>
+      <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FBA79585</t>
+          <t>FBA77101</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>B0CFKHCQ8W</t>
+          <t>B07WLWN2ZT</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2020,25 +2020,25 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>T20LP</t>
+          <t>TC-777</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Low Profile Boom Arm</t>
+          <t>Tripod</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>845</v>
+        <v>1206</v>
       </c>
       <c r="I25" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -2050,32 +2050,32 @@
         <v>24</v>
       </c>
       <c r="M25" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N25" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="O25" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="P25" t="n">
-        <v>2922.69</v>
+        <v>66812.92</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FBA79111</t>
+          <t>FBA77115</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>B0BRKFP94K</t>
+          <t>B08V1JS3NY</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2085,25 +2085,25 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>TD510</t>
+          <t>TC40</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Dynamic Microphone</t>
+          <t>Condenser Microphone</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>USB/XLR Mic</t>
+          <t>Boom Arm Kit - USB</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>2412</v>
+        <v>1930</v>
       </c>
       <c r="I26" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -2115,32 +2115,32 @@
         <v>24</v>
       </c>
       <c r="M26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N26" t="n">
         <v>2</v>
       </c>
       <c r="O26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P26" t="n">
-        <v>21992.2</v>
+        <v>22543.15</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FBA77104</t>
+          <t>FBA77116</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>B089SJGQBH</t>
+          <t>B0BBL47VR5</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>TC20</t>
+          <t>TC40S</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2160,15 +2160,15 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Boom Arm Kit - XLR</t>
+          <t>Boom Arm Kit - USB - RGB</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>3015</v>
+        <v>1930</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -2180,18 +2180,20 @@
         <v>24</v>
       </c>
       <c r="M27" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="P27" t="n">
+        <v>10345.5</v>
+      </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2233,7 @@
         <v>1327</v>
       </c>
       <c r="I28" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -2246,29 +2248,29 @@
         <v>52</v>
       </c>
       <c r="N28" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O28" t="n">
         <v>4</v>
       </c>
       <c r="P28" t="n">
-        <v>88083.5</v>
+        <v>86332.34</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>FBA79113</t>
+          <t>FBK77102</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>B0BTCXQQ6M</t>
+          <t>B07GVGMW59</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2278,25 +2280,25 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>TC310</t>
+          <t>G11</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Condenser Microphone</t>
+          <t>Conference Microphone</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Tripod - RGB</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>1206</v>
+        <v>1108</v>
       </c>
       <c r="I29" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2308,32 +2310,32 @@
         <v>24</v>
       </c>
       <c r="M29" t="n">
+        <v>18</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
         <v>3</v>
       </c>
-      <c r="N29" t="n">
-        <v>1</v>
-      </c>
-      <c r="O29" t="n">
-        <v>2</v>
-      </c>
       <c r="P29" t="n">
-        <v>28018.53</v>
+        <v>94093.78999999999</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FBA79582</t>
+          <t>FBA79112</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>B0CCVBQRFX</t>
+          <t>B0BRKDLXCD</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2343,25 +2345,25 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>TD510+</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Dynamic Microphone</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Hand held Mic + Boom Arm</t>
+          <t>Boom Arm - RGB</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>3491</v>
+        <v>2412</v>
       </c>
       <c r="I30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -2381,12 +2383,10 @@
       <c r="O30" t="n">
         <v>0</v>
       </c>
-      <c r="P30" t="n">
-        <v>4334.39</v>
-      </c>
+      <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>

</xml_diff>